<commit_message>
feat: contexto institucional en system prompts + 7 estudiantes dummies
- prompts.py: bloque CONTEXTO INSTITUCIONAL en TUTOR_SYSTEM_PROMPT y
  DEGRADED_RESPONSE_SYSTEM_PROMPT (descripción del Colombo Americano Cali,
  misión de LIA, ciclos Fundamental / Fundamental Plus / Pre-Independent /
  Independent).
- estudiantes_dummies.xlsx: agregados 7 estudiantes Fundamental Plus (No.
  6-12) para ampliar pool de prueba con usuarios reales. Todos en estado
  Pass, debilidades variadas en teacher_feedback.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/user/estudiantes_dummies.xlsx
+++ b/data/user/estudiantes_dummies.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -721,6 +721,293 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>inv88p12</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Fundamental Plus 2</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1133445566</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>TORRES PINEDA ANDREA MILENA</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>atorres@t.colomboamericano.edu.co</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>78</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>"Good progress overall! Focus on irregular past simple verbs (go/went, see/saw, take/took). Practice narrating past events using a wider verb range."</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>inv88p12</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Fundamental Plus 5</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1177889900</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>VARGAS MORA CARLOS ANDRES</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>cvargas@t.colomboamericano.edu.co</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>74</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>"You need to work on Present Perfect with since and for. You often confuse it with Simple Past. Practice time expressions: I have lived here since 2010 / for five years."</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>inv88p12</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Fundamental Plus 8</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1166778899</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>PRADO SALCEDO LUISA FERNANDA</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>lprado@t.colomboamericano.edu.co</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>88</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>"Excellent reading comprehension! To reach the next level, work on modal verbs of obligation: must, have to, should. Practice distinguishing strong obligation from advice."</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>inv88p12</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Fundamental Plus 11</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1188990011</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>MORALES GUERRERO ESTEBAN</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>emorales@t.colomboamericano.edu.co</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>73</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>"Good spoken fluency. However, pronunciation of -ed endings needs work: /t/ (walked), /d/ (played), /id/ (wanted). Dedicate 10 min a day to minimal pairs practice."</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>inv88p12</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Fundamental Plus 3</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1155443322</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>CORREA LONDONO NATALIA ISABEL</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>ncorrea@t.colomboamericano.edu.co</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>80</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>"You are communicative and motivated! Please review travel and transportation vocabulary (Unit 9). Practice using prepositions of movement: across, through, along, past."</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>inv88p12</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Fundamental Plus 6</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1199001122</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>GUTIERREZ LOZANO MIGUEL ANGEL</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>mgutierrez@t.colomboamericano.edu.co</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>71</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>"Review Present Continuous vs Simple Present. You frequently use present continuous for habits. Remember: I work every day (habit) vs I am working right now (action in progress)."</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>inv88p12</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Fundamental Plus 9</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1122110033</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>SILVA CAMACHO DIANA CAROLINA</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>dsilva@t.colomboamericano.edu.co</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>81</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>"Great written accuracy! For next cycle, focus on comparatives and superlatives in extended discourse. Practice comparing options in real-life situations: jobs, cities, routines."</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>